<commit_message>
added band-power ratio features (4); 140 total now (up from 86)
</commit_message>
<xml_diff>
--- a/data/model_results.xlsx
+++ b/data/model_results.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="13.57142857142857" customWidth="1" min="1" max="24"/>
@@ -1453,6 +1453,231 @@
       </c>
       <c r="K22" t="n">
         <v>0.0309128996279603</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>EXP022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>3-class</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>all 84</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>gradient_boosting</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0.4265442764578833</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.02004598922973724</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.3397535531599024</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.0298790806979595</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.3618156095126175</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0.01789576306457959</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>EXP023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>all 84</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>dummy</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>0.478823326538037</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.03370685959152283</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.3234278522102419</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.01574589215118924</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>EXP024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>all 84</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>logistic_regression</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>0.56642439534036</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.03670335116016884</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.5597804620088429</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.03660267641305567</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.5729175336275398</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0.03098413221474304</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>EXP025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>all 84</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>lda</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>0.5781996722413855</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.02805468125320993</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.5735126492851343</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.02621384814996985</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.5829619057495343</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0.02650448303414387</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>EXP026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>all 140</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>gradient_boosting</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>0.5862980816024456</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.02584931430138216</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.582556344556848</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.02577308142663746</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.5843584712701475</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0.02416365815710252</v>
       </c>
     </row>
   </sheetData>
@@ -1467,7 +1692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="13.57142857142857" customWidth="1" min="1" max="24"/>
@@ -3780,6 +4005,481 @@
         <v>0.4244291267007392</v>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>EXP022</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>1</v>
+      </c>
+      <c r="C122" t="n">
+        <v>0.3995680345572354</v>
+      </c>
+      <c r="D122" t="n">
+        <v>0.3089544274618323</v>
+      </c>
+      <c r="E122" t="n">
+        <v>0.3383576587478707</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>EXP022</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>2</v>
+      </c>
+      <c r="C123" t="n">
+        <v>0.4319654427645788</v>
+      </c>
+      <c r="D123" t="n">
+        <v>0.3270215757609074</v>
+      </c>
+      <c r="E123" t="n">
+        <v>0.3460216957734</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>EXP022</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>3</v>
+      </c>
+      <c r="C124" t="n">
+        <v>0.406695464362851</v>
+      </c>
+      <c r="D124" t="n">
+        <v>0.3116766154056929</v>
+      </c>
+      <c r="E124" t="n">
+        <v>0.3619408744436232</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>EXP022</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>4</v>
+      </c>
+      <c r="C125" t="n">
+        <v>0.4465442764578834</v>
+      </c>
+      <c r="D125" t="n">
+        <v>0.3762423120718287</v>
+      </c>
+      <c r="E125" t="n">
+        <v>0.3856278753298186</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>EXP022</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>5</v>
+      </c>
+      <c r="C126" t="n">
+        <v>0.4479481641468683</v>
+      </c>
+      <c r="D126" t="n">
+        <v>0.3748728350992502</v>
+      </c>
+      <c r="E126" t="n">
+        <v>0.3771299432683753</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>EXP023</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>1</v>
+      </c>
+      <c r="C127" t="n">
+        <v>0.4668129456939111</v>
+      </c>
+      <c r="D127" t="n">
+        <v>0.3182498130142109</v>
+      </c>
+      <c r="E127" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>EXP023</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>2</v>
+      </c>
+      <c r="C128" t="n">
+        <v>0.5097122302158273</v>
+      </c>
+      <c r="D128" t="n">
+        <v>0.3376221110316893</v>
+      </c>
+      <c r="E128" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>EXP023</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>3</v>
+      </c>
+      <c r="C129" t="n">
+        <v>0.5056717922863625</v>
+      </c>
+      <c r="D129" t="n">
+        <v>0.3358446341871756</v>
+      </c>
+      <c r="E129" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>EXP023</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>4</v>
+      </c>
+      <c r="C130" t="n">
+        <v>0.4184360435007768</v>
+      </c>
+      <c r="D130" t="n">
+        <v>0.2949981745162468</v>
+      </c>
+      <c r="E130" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>EXP023</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>5</v>
+      </c>
+      <c r="C131" t="n">
+        <v>0.4934836209933075</v>
+      </c>
+      <c r="D131" t="n">
+        <v>0.3304245283018868</v>
+      </c>
+      <c r="E131" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>EXP024</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>1</v>
+      </c>
+      <c r="C132" t="n">
+        <v>0.6226001097092705</v>
+      </c>
+      <c r="D132" t="n">
+        <v>0.6223159939882481</v>
+      </c>
+      <c r="E132" t="n">
+        <v>0.6271836449976547</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>EXP024</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>2</v>
+      </c>
+      <c r="C133" t="n">
+        <v>0.5496402877697841</v>
+      </c>
+      <c r="D133" t="n">
+        <v>0.5474363795326447</v>
+      </c>
+      <c r="E133" t="n">
+        <v>0.5512037821837441</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>EXP024</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>3</v>
+      </c>
+      <c r="C134" t="n">
+        <v>0.5903705570960424</v>
+      </c>
+      <c r="D134" t="n">
+        <v>0.5708531437172887</v>
+      </c>
+      <c r="E134" t="n">
+        <v>0.5880270966803821</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>EXP024</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>4</v>
+      </c>
+      <c r="C135" t="n">
+        <v>0.5157949249093734</v>
+      </c>
+      <c r="D135" t="n">
+        <v>0.5113094039413881</v>
+      </c>
+      <c r="E135" t="n">
+        <v>0.5459516037311657</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>EXP024</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>5</v>
+      </c>
+      <c r="C136" t="n">
+        <v>0.5537160972173301</v>
+      </c>
+      <c r="D136" t="n">
+        <v>0.5469873888646452</v>
+      </c>
+      <c r="E136" t="n">
+        <v>0.552221540544753</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>EXP025</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>1</v>
+      </c>
+      <c r="C137" t="n">
+        <v>0.6162918266593527</v>
+      </c>
+      <c r="D137" t="n">
+        <v>0.6162737853456459</v>
+      </c>
+      <c r="E137" t="n">
+        <v>0.6194760581837877</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>EXP025</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>2</v>
+      </c>
+      <c r="C138" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D138" t="n">
+        <v>0.5499202733883169</v>
+      </c>
+      <c r="E138" t="n">
+        <v>0.5499489740707508</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>EXP025</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>3</v>
+      </c>
+      <c r="C139" t="n">
+        <v>0.608016133098059</v>
+      </c>
+      <c r="D139" t="n">
+        <v>0.5919991100112949</v>
+      </c>
+      <c r="E139" t="n">
+        <v>0.6058465348472686</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>EXP025</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>4</v>
+      </c>
+      <c r="C140" t="n">
+        <v>0.5559295701708959</v>
+      </c>
+      <c r="D140" t="n">
+        <v>0.5546252216424279</v>
+      </c>
+      <c r="E140" t="n">
+        <v>0.5801970279396595</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>EXP025</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>5</v>
+      </c>
+      <c r="C141" t="n">
+        <v>0.5607608312786192</v>
+      </c>
+      <c r="D141" t="n">
+        <v>0.5547448560379855</v>
+      </c>
+      <c r="E141" t="n">
+        <v>0.5593409337062043</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>EXP026</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>1</v>
+      </c>
+      <c r="C142" t="n">
+        <v>0.5806363137685134</v>
+      </c>
+      <c r="D142" t="n">
+        <v>0.5775227434337271</v>
+      </c>
+      <c r="E142" t="n">
+        <v>0.5774823736780259</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>EXP026</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>2</v>
+      </c>
+      <c r="C143" t="n">
+        <v>0.5636690647482014</v>
+      </c>
+      <c r="D143" t="n">
+        <v>0.5616858070216006</v>
+      </c>
+      <c r="E143" t="n">
+        <v>0.5625747202375928</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>EXP026</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>3</v>
+      </c>
+      <c r="C144" t="n">
+        <v>0.6135618855558357</v>
+      </c>
+      <c r="D144" t="n">
+        <v>0.6134954750376325</v>
+      </c>
+      <c r="E144" t="n">
+        <v>0.6137895594196503</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>EXP026</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>4</v>
+      </c>
+      <c r="C145" t="n">
+        <v>0.6188503366131538</v>
+      </c>
+      <c r="D145" t="n">
+        <v>0.6107832529138209</v>
+      </c>
+      <c r="E145" t="n">
+        <v>0.6116415431614399</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>EXP026</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>5</v>
+      </c>
+      <c r="C146" t="n">
+        <v>0.5547728073265235</v>
+      </c>
+      <c r="D146" t="n">
+        <v>0.5492944443774592</v>
+      </c>
+      <c r="E146" t="n">
+        <v>0.5563041598540284</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>

<commit_message>
ran tests on 140 features
</commit_message>
<xml_diff>
--- a/data/model_results.xlsx
+++ b/data/model_results.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="13.57142857142857" customWidth="1" min="1" max="24"/>
@@ -1678,6 +1678,141 @@
       </c>
       <c r="K27" t="n">
         <v>0.02416365815710252</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>EXP027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>all 140</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>random_forest</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>0.5738774346411954</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.0345374109384961</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.5679262488643964</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0.03401045500660053</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.5728264113425471</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0.03376886378812451</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>EXP028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>5-class</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>all 140</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>rbf_svm</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>0.2387041036717063</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.0390453274590896</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.2221315403225575</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.04058974785039939</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.2396131216387739</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0.03752713934767387</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>EXP029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>3-class</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>all 140</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>linear_svm</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>0.4408207343412527</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.0433020310269277</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.343536860342837</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0.02693314179970802</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.3737431083279039</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0.02112229237330866</v>
       </c>
     </row>
   </sheetData>
@@ -1692,7 +1827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E146"/>
+  <dimension ref="A1:E161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="13.57142857142857" customWidth="1" min="1" max="24"/>
@@ -4480,6 +4615,291 @@
         <v>0.5563041598540284</v>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>EXP027</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>1</v>
+      </c>
+      <c r="C147" t="n">
+        <v>0.6091607240811848</v>
+      </c>
+      <c r="D147" t="n">
+        <v>0.5993337073517759</v>
+      </c>
+      <c r="E147" t="n">
+        <v>0.6014154250869227</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>EXP027</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>2</v>
+      </c>
+      <c r="C148" t="n">
+        <v>0.5298561151079136</v>
+      </c>
+      <c r="D148" t="n">
+        <v>0.5191403057764015</v>
+      </c>
+      <c r="E148" t="n">
+        <v>0.5271553212717806</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>EXP027</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>3</v>
+      </c>
+      <c r="C149" t="n">
+        <v>0.6112931686412907</v>
+      </c>
+      <c r="D149" t="n">
+        <v>0.6040924313358786</v>
+      </c>
+      <c r="E149" t="n">
+        <v>0.6098418157053571</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>EXP027</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>4</v>
+      </c>
+      <c r="C150" t="n">
+        <v>0.5815639564992232</v>
+      </c>
+      <c r="D150" t="n">
+        <v>0.5801261143726897</v>
+      </c>
+      <c r="E150" t="n">
+        <v>0.5876558325912733</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>EXP027</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>5</v>
+      </c>
+      <c r="C151" t="n">
+        <v>0.5375132088763649</v>
+      </c>
+      <c r="D151" t="n">
+        <v>0.5369386854852365</v>
+      </c>
+      <c r="E151" t="n">
+        <v>0.538063662057402</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>EXP028</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>1</v>
+      </c>
+      <c r="C152" t="n">
+        <v>0.3092872570194384</v>
+      </c>
+      <c r="D152" t="n">
+        <v>0.29607680020081</v>
+      </c>
+      <c r="E152" t="n">
+        <v>0.3056564411531211</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>EXP028</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>2</v>
+      </c>
+      <c r="C153" t="n">
+        <v>0.2224622030237581</v>
+      </c>
+      <c r="D153" t="n">
+        <v>0.2053710688960955</v>
+      </c>
+      <c r="E153" t="n">
+        <v>0.2184881941371026</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>EXP028</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>3</v>
+      </c>
+      <c r="C154" t="n">
+        <v>0.2131749460043197</v>
+      </c>
+      <c r="D154" t="n">
+        <v>0.1836558312111981</v>
+      </c>
+      <c r="E154" t="n">
+        <v>0.2064326470452619</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>EXP028</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>4</v>
+      </c>
+      <c r="C155" t="n">
+        <v>0.1987041036717063</v>
+      </c>
+      <c r="D155" t="n">
+        <v>0.1923634233642937</v>
+      </c>
+      <c r="E155" t="n">
+        <v>0.2106832102520648</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>EXP028</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>5</v>
+      </c>
+      <c r="C156" t="n">
+        <v>0.2498920086393089</v>
+      </c>
+      <c r="D156" t="n">
+        <v>0.2331905779403902</v>
+      </c>
+      <c r="E156" t="n">
+        <v>0.2568051156063189</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>EXP029</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>1</v>
+      </c>
+      <c r="C157" t="n">
+        <v>0.3876889848812095</v>
+      </c>
+      <c r="D157" t="n">
+        <v>0.3037685140696251</v>
+      </c>
+      <c r="E157" t="n">
+        <v>0.3437718557938051</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>EXP029</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>2</v>
+      </c>
+      <c r="C158" t="n">
+        <v>0.4254859611231102</v>
+      </c>
+      <c r="D158" t="n">
+        <v>0.347864579660899</v>
+      </c>
+      <c r="E158" t="n">
+        <v>0.3682495835996573</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>EXP029</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>3</v>
+      </c>
+      <c r="C159" t="n">
+        <v>0.438012958963283</v>
+      </c>
+      <c r="D159" t="n">
+        <v>0.3432123674416916</v>
+      </c>
+      <c r="E159" t="n">
+        <v>0.3845329766236599</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>EXP029</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>4</v>
+      </c>
+      <c r="C160" t="n">
+        <v>0.4330453563714903</v>
+      </c>
+      <c r="D160" t="n">
+        <v>0.3350846246442535</v>
+      </c>
+      <c r="E160" t="n">
+        <v>0.3650870571603957</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>EXP029</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>5</v>
+      </c>
+      <c r="C161" t="n">
+        <v>0.5198704103671706</v>
+      </c>
+      <c r="D161" t="n">
+        <v>0.3877542158977159</v>
+      </c>
+      <c r="E161" t="n">
+        <v>0.4070740684620016</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>